<commit_message>
This is the commit for both this and the privous week. I spent most of the time writting down the Research Horizons article and ordering my results in a paper format in order to sort the ideas out so I can get a more coherent story. Apart from that, the main code being backed up is the one used for processing gridded ARGO data and computing stratification variables (MLD and N2 (haline and thermal components)). Next weel I'll go to London for the ARIA training week so I'll probably won't be updating the code.
</commit_message>
<xml_diff>
--- a/notebooks/OMP_stuff_for_Manuel/RREX_WMTYPES_5poly_ORIGINAL.xlsx
+++ b/notebooks/OMP_stuff_for_Manuel/RREX_WMTYPES_5poly_ORIGINAL.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399BF978-767B-4FC1-9116-18305CB7D5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="10690" windowWidth="19420" windowHeight="11500" xr2:uid="{55C3EF8E-6B26-4C61-893E-38A87239426C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{55C3EF8E-6B26-4C61-893E-38A87239426C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -474,16 +474,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5534A5F-E9E6-40C7-9BD6-42148A7D753A}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
-    <col min="7" max="7" width="32.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.7265625" customWidth="1"/>
+    <col min="7" max="7" width="32.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -498,7 +498,7 @@
       </c>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -521,7 +521,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -544,7 +544,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -567,7 +567,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -590,7 +590,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -610,7 +610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -630,7 +630,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -653,49 +653,49 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>

</xml_diff>